<commit_message>
Update embedded bw-amr-ig with rebuilt IG including all new artifacts
Rebuilt IG now includes Encounter profile, AST method/ward type ValueSets,
$export-whonet OperationDefinition, 23 example instances, and updated
narrative pages. ConceptMaps excluded from publisher build (used by
export package, not needed in rendered IG).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/static/bw_amr_ig/StructureDefinition-botswana-amr-diagnostic-report.xlsx
+++ b/static/bw_amr_ig/StructureDefinition-botswana-amr-diagnostic-report.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1710" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1670" uniqueCount="394">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-07-09T10:14:37-04:00</t>
+    <t>2026-03-13T15:05:11-04:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -81,7 +81,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Bundles AMR susceptibility observations into one comprehensive report</t>
+    <t>Bundles AMR culture results into one comprehensive report. References top-level observations (gram stain and organism identifications). Susceptibility and special test results are accessed via OrganismObservation.hasMember.</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -439,7 +439,7 @@
     <t>DiagnosticReport.meta.profile</t>
   </si>
   <si>
-    <t xml:space="preserve">canonical(StructureDefinition)
+    <t xml:space="preserve">canonical(StructureDefinition|4.3.0)
 </t>
   </si>
   <si>
@@ -477,7 +477,7 @@
     <t>extensible</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/security-labels</t>
+    <t>http://hl7.org/fhir/ValueSet/security-labels|4.3.0</t>
   </si>
   <si>
     <t>Meta.security</t>
@@ -498,7 +498,7 @@
     <t>example</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/common-tags</t>
+    <t>http://hl7.org/fhir/ValueSet/common-tags|4.3.0</t>
   </si>
   <si>
     <t>Meta.tag</t>
@@ -541,7 +541,7 @@
     <t>IETF language tag</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/languages</t>
+    <t>http://hl7.org/fhir/ValueSet/languages|4.3.0</t>
   </si>
   <si>
     <t>Resource.language</t>
@@ -670,7 +670,7 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(CarePlan|ImmunizationRecommendation|MedicationRequest|NutritionOrder|ServiceRequest)
+    <t xml:space="preserve">Reference(CarePlan|4.3.0|ImmunizationRecommendation|4.3.0|MedicationRequest|4.3.0|NutritionOrder|4.3.0|ServiceRequest|4.3.0)
 </t>
   </si>
   <si>
@@ -751,7 +751,11 @@
     <t>HL7 V2 table 0074</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/diagnostic-service-sections</t>
+    <t>http://hl7.org/fhir/ValueSet/diagnostic-service-sections|4.3.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pattern:$this}
+</t>
   </si>
   <si>
     <t>OBR-24</t>
@@ -761,6 +765,21 @@
   </si>
   <si>
     <t>FiveWs.class</t>
+  </si>
+  <si>
+    <t>DiagnosticReport.category:microbiologyStudies</t>
+  </si>
+  <si>
+    <t>microbiologyStudies</t>
+  </si>
+  <si>
+    <t>&lt;valueCodeableConcept xmlns="http://hl7.org/fhir"&gt;
+  &lt;coding&gt;
+    &lt;system value="http://loinc.org"/&gt;
+    &lt;code value="18725-2"/&gt;
+    &lt;display value="Microbiology studies (set)"/&gt;
+  &lt;/coding&gt;
+&lt;/valueCodeableConcept&gt;</t>
   </si>
   <si>
     <t>DiagnosticReport.code</t>
@@ -788,7 +807,7 @@
     <t>LOINC Codes for Diagnostic Reports</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/report-codes</t>
+    <t>http://hl7.org/fhir/ValueSet/report-codes|4.3.0</t>
   </si>
   <si>
     <t>Event.code</t>
@@ -842,7 +861,7 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Encounter)
+    <t xml:space="preserve">Reference(http://bw.health.gov/fhir/ImplementationGuide/bw-amr-ig/StructureDefinition/botswana-amr-encounter)
 </t>
   </si>
   <si>
@@ -953,7 +972,7 @@
 ServicePractitionerDepartmentCompanyAuthorized byDirector</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Practitioner|PractitionerRole|Organization|CareTeam)
+    <t xml:space="preserve">Reference(Organization|Practitioner)
 </t>
   </si>
   <si>
@@ -988,6 +1007,10 @@
 Reported by</t>
   </si>
   <si>
+    <t xml:space="preserve">Reference(Practitioner|4.3.0|PractitionerRole|4.3.0|Organization|4.3.0|CareTeam|4.3.0)
+</t>
+  </si>
+  <si>
     <t>Primary result interpreter</t>
   </si>
   <si>
@@ -1029,7 +1052,7 @@
 Atomic ValueResultAtomic resultDataTestAnalyteBatteryOrganizer</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Observation)
+    <t xml:space="preserve">Reference(Observation|4.3.0)
 </t>
   </si>
   <si>
@@ -1075,30 +1098,10 @@
 </t>
   </si>
   <si>
-    <t>DiagnosticReport.result:susceptibility</t>
-  </si>
-  <si>
-    <t>susceptibility</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference(http://bw.health.gov/fhir/ImplementationGuide/bw-amr-ig/StructureDefinition/botswana-amr-susceptibility-observation)
-</t>
-  </si>
-  <si>
-    <t>DiagnosticReport.result:specialTests</t>
-  </si>
-  <si>
-    <t>specialTests</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference(http://bw.health.gov/fhir/ImplementationGuide/bw-amr-ig/StructureDefinition/botswana-amr-special-test-observation)
-</t>
-  </si>
-  <si>
     <t>DiagnosticReport.imagingStudy</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(ImagingStudy)
+    <t xml:space="preserve">Reference(ImagingStudy|4.3.0)
 </t>
   </si>
   <si>
@@ -1189,7 +1192,7 @@
     <t>DiagnosticReport.media.link</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Media)
+    <t xml:space="preserve">Reference(Media|4.3.0)
 </t>
   </si>
   <si>
@@ -1236,7 +1239,7 @@
     <t>SNOMED CT Clinical Findings</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/clinical-findings</t>
+    <t>http://hl7.org/fhir/ValueSet/clinical-findings|4.3.0</t>
   </si>
   <si>
     <t>inboundRelationship[typeCode=SPRT].source[classCode=OBS, moodCode=EVN, code=LOINC:54531-9].value (type=CD)</t>
@@ -1563,12 +1566,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AN46"/>
+  <dimension ref="A1:AN45"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="40.0234375" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="40.05859375" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="36.21875" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="15.80078125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="3" max="3" width="17.69921875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="55.23046875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.65234375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.265625" customWidth="true" bestFit="true"/>
@@ -1576,7 +1579,7 @@
     <col min="8" max="8" width="13.609375" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.1796875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="108.9453125" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="112.67578125" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -1591,7 +1594,7 @@
     <col min="23" max="23" width="16.40625" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="15.85546875" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="30.55859375" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="48.58203125" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="50.8203125" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.2734375" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.55859375" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="36.56640625" customWidth="true" bestFit="true"/>
@@ -4020,7 +4023,7 @@
       </c>
       <c r="E22" s="2"/>
       <c r="F22" t="s" s="2">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="G22" t="s" s="2">
         <v>79</v>
@@ -4082,16 +4085,14 @@
         <v>20</v>
       </c>
       <c r="AB22" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AC22" t="s" s="2">
-        <v>20</v>
-      </c>
+        <v>237</v>
+      </c>
+      <c r="AC22" s="2"/>
       <c r="AD22" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AE22" t="s" s="2">
-        <v>20</v>
+        <v>116</v>
       </c>
       <c r="AF22" t="s" s="2">
         <v>229</v>
@@ -4112,25 +4113,27 @@
         <v>20</v>
       </c>
       <c r="AL22" t="s" s="2">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="AM22" t="s" s="2">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="AN22" t="s" s="2">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>240</v>
-      </c>
-      <c r="C23" s="2"/>
+        <v>229</v>
+      </c>
+      <c r="C23" t="s" s="2">
+        <v>242</v>
+      </c>
       <c r="D23" t="s" s="2">
-        <v>241</v>
+        <v>230</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
@@ -4152,12 +4155,14 @@
         <v>231</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>243</v>
-      </c>
-      <c r="N23" s="2"/>
+        <v>233</v>
+      </c>
+      <c r="N23" t="s" s="2">
+        <v>234</v>
+      </c>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
         <v>20</v>
@@ -4167,7 +4172,7 @@
         <v>20</v>
       </c>
       <c r="S23" t="s" s="2">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="T23" t="s" s="2">
         <v>20</v>
@@ -4182,13 +4187,13 @@
         <v>20</v>
       </c>
       <c r="X23" t="s" s="2">
-        <v>168</v>
+        <v>155</v>
       </c>
       <c r="Y23" t="s" s="2">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="Z23" t="s" s="2">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>20</v>
@@ -4206,13 +4211,13 @@
         <v>20</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>240</v>
+        <v>229</v>
       </c>
       <c r="AG23" t="s" s="2">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="AH23" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="AI23" t="s" s="2">
         <v>20</v>
@@ -4221,28 +4226,28 @@
         <v>102</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>247</v>
+        <v>20</v>
       </c>
       <c r="AL23" t="s" s="2">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="AM23" t="s" s="2">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="AN23" t="s" s="2">
-        <v>250</v>
+        <v>240</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" t="s" s="2">
@@ -4261,18 +4266,16 @@
         <v>91</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>253</v>
+        <v>231</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="N24" s="2"/>
-      <c r="O24" t="s" s="2">
-        <v>256</v>
-      </c>
+      <c r="O24" s="2"/>
       <c r="P24" t="s" s="2">
         <v>20</v>
       </c>
@@ -4281,7 +4284,7 @@
         <v>20</v>
       </c>
       <c r="S24" t="s" s="2">
-        <v>20</v>
+        <v>248</v>
       </c>
       <c r="T24" t="s" s="2">
         <v>20</v>
@@ -4296,13 +4299,13 @@
         <v>20</v>
       </c>
       <c r="X24" t="s" s="2">
-        <v>20</v>
+        <v>168</v>
       </c>
       <c r="Y24" t="s" s="2">
-        <v>20</v>
+        <v>249</v>
       </c>
       <c r="Z24" t="s" s="2">
-        <v>20</v>
+        <v>250</v>
       </c>
       <c r="AA24" t="s" s="2">
         <v>20</v>
@@ -4320,10 +4323,10 @@
         <v>20</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="AG24" t="s" s="2">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="AH24" t="s" s="2">
         <v>90</v>
@@ -4335,32 +4338,32 @@
         <v>102</v>
       </c>
       <c r="AK24" t="s" s="2">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="AL24" t="s" s="2">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="AM24" t="s" s="2">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="AN24" t="s" s="2">
-        <v>260</v>
+        <v>254</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" t="s" s="2">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="G25" t="s" s="2">
         <v>90</v>
@@ -4375,19 +4378,17 @@
         <v>91</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>265</v>
-      </c>
-      <c r="N25" t="s" s="2">
-        <v>266</v>
-      </c>
+        <v>259</v>
+      </c>
+      <c r="N25" s="2"/>
       <c r="O25" t="s" s="2">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="P25" t="s" s="2">
         <v>20</v>
@@ -4436,7 +4437,7 @@
         <v>20</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>78</v>
@@ -4451,32 +4452,32 @@
         <v>102</v>
       </c>
       <c r="AK25" t="s" s="2">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="AL25" t="s" s="2">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="AM25" t="s" s="2">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="AN25" t="s" s="2">
-        <v>271</v>
+        <v>264</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="E26" s="2"/>
       <c r="F26" t="s" s="2">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="G26" t="s" s="2">
         <v>90</v>
@@ -4491,19 +4492,19 @@
         <v>91</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="N26" t="s" s="2">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="O26" t="s" s="2">
-        <v>278</v>
+        <v>271</v>
       </c>
       <c r="P26" t="s" s="2">
         <v>20</v>
@@ -4540,17 +4541,19 @@
         <v>20</v>
       </c>
       <c r="AB26" t="s" s="2">
-        <v>279</v>
-      </c>
-      <c r="AC26" s="2"/>
+        <v>20</v>
+      </c>
+      <c r="AC26" t="s" s="2">
+        <v>20</v>
+      </c>
       <c r="AD26" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AE26" t="s" s="2">
-        <v>280</v>
+        <v>20</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>78</v>
@@ -4565,30 +4568,28 @@
         <v>102</v>
       </c>
       <c r="AK26" t="s" s="2">
-        <v>281</v>
+        <v>272</v>
       </c>
       <c r="AL26" t="s" s="2">
-        <v>282</v>
+        <v>273</v>
       </c>
       <c r="AM26" t="s" s="2">
-        <v>283</v>
+        <v>274</v>
       </c>
       <c r="AN26" t="s" s="2">
-        <v>284</v>
+        <v>275</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>285</v>
+        <v>276</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>272</v>
-      </c>
-      <c r="C27" t="s" s="2">
-        <v>286</v>
-      </c>
+        <v>276</v>
+      </c>
+      <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" t="s" s="2">
@@ -4607,19 +4608,19 @@
         <v>91</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="N27" t="s" s="2">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="O27" t="s" s="2">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="P27" t="s" s="2">
         <v>20</v>
@@ -4656,19 +4657,17 @@
         <v>20</v>
       </c>
       <c r="AB27" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AC27" t="s" s="2">
-        <v>20</v>
-      </c>
+        <v>283</v>
+      </c>
+      <c r="AC27" s="2"/>
       <c r="AD27" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AE27" t="s" s="2">
-        <v>20</v>
+        <v>284</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>78</v>
@@ -4683,32 +4682,34 @@
         <v>102</v>
       </c>
       <c r="AK27" t="s" s="2">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="AL27" t="s" s="2">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="AM27" t="s" s="2">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="AN27" t="s" s="2">
-        <v>284</v>
+        <v>288</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>287</v>
-      </c>
-      <c r="C28" s="2"/>
+        <v>276</v>
+      </c>
+      <c r="C28" t="s" s="2">
+        <v>290</v>
+      </c>
       <c r="D28" t="s" s="2">
-        <v>288</v>
+        <v>277</v>
       </c>
       <c r="E28" s="2"/>
       <c r="F28" t="s" s="2">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="G28" t="s" s="2">
         <v>90</v>
@@ -4723,19 +4724,19 @@
         <v>91</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>125</v>
+        <v>278</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>289</v>
+        <v>279</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>290</v>
+        <v>280</v>
       </c>
       <c r="N28" t="s" s="2">
-        <v>291</v>
+        <v>281</v>
       </c>
       <c r="O28" t="s" s="2">
-        <v>292</v>
+        <v>282</v>
       </c>
       <c r="P28" t="s" s="2">
         <v>20</v>
@@ -4784,7 +4785,7 @@
         <v>20</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>287</v>
+        <v>276</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>78</v>
@@ -4799,35 +4800,35 @@
         <v>102</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>20</v>
+        <v>285</v>
       </c>
       <c r="AL28" t="s" s="2">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="AM28" t="s" s="2">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="AN28" t="s" s="2">
-        <v>295</v>
+        <v>288</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G29" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="H29" t="s" s="2">
         <v>20</v>
@@ -4839,19 +4840,19 @@
         <v>91</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>298</v>
+        <v>125</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>299</v>
+        <v>293</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>300</v>
+        <v>294</v>
       </c>
       <c r="N29" t="s" s="2">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="O29" t="s" s="2">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="P29" t="s" s="2">
         <v>20</v>
@@ -4900,13 +4901,13 @@
         <v>20</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH29" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="AI29" t="s" s="2">
         <v>20</v>
@@ -4915,28 +4916,28 @@
         <v>102</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>303</v>
+        <v>20</v>
       </c>
       <c r="AL29" t="s" s="2">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="AM29" t="s" s="2">
-        <v>305</v>
+        <v>298</v>
       </c>
       <c r="AN29" t="s" s="2">
-        <v>306</v>
+        <v>299</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" t="s" s="2">
@@ -4955,19 +4956,19 @@
         <v>91</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="N30" t="s" s="2">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="O30" t="s" s="2">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="P30" t="s" s="2">
         <v>20</v>
@@ -5016,7 +5017,7 @@
         <v>20</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>78</v>
@@ -5031,32 +5032,32 @@
         <v>102</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="AM30" t="s" s="2">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="AN30" t="s" s="2">
-        <v>306</v>
+        <v>310</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
-        <v>20</v>
+        <v>312</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s" s="2">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="G31" t="s" s="2">
         <v>79</v>
@@ -5068,22 +5069,22 @@
         <v>20</v>
       </c>
       <c r="J31" t="s" s="2">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="K31" t="s" s="2">
+        <v>313</v>
+      </c>
+      <c r="L31" t="s" s="2">
         <v>314</v>
       </c>
-      <c r="L31" t="s" s="2">
+      <c r="M31" t="s" s="2">
         <v>315</v>
       </c>
-      <c r="M31" t="s" s="2">
+      <c r="N31" t="s" s="2">
         <v>316</v>
       </c>
-      <c r="N31" t="s" s="2">
-        <v>317</v>
-      </c>
       <c r="O31" t="s" s="2">
-        <v>318</v>
+        <v>306</v>
       </c>
       <c r="P31" t="s" s="2">
         <v>20</v>
@@ -5132,7 +5133,7 @@
         <v>20</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>78</v>
@@ -5147,28 +5148,28 @@
         <v>102</v>
       </c>
       <c r="AK31" t="s" s="2">
-        <v>20</v>
+        <v>307</v>
       </c>
       <c r="AL31" t="s" s="2">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="AM31" t="s" s="2">
-        <v>259</v>
+        <v>309</v>
       </c>
       <c r="AN31" t="s" s="2">
-        <v>20</v>
+        <v>310</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
-        <v>321</v>
+        <v>20</v>
       </c>
       <c r="E32" s="2"/>
       <c r="F32" t="s" s="2">
@@ -5187,19 +5188,19 @@
         <v>20</v>
       </c>
       <c r="K32" t="s" s="2">
+        <v>319</v>
+      </c>
+      <c r="L32" t="s" s="2">
+        <v>320</v>
+      </c>
+      <c r="M32" t="s" s="2">
+        <v>321</v>
+      </c>
+      <c r="N32" t="s" s="2">
         <v>322</v>
       </c>
-      <c r="L32" t="s" s="2">
+      <c r="O32" t="s" s="2">
         <v>323</v>
-      </c>
-      <c r="M32" t="s" s="2">
-        <v>324</v>
-      </c>
-      <c r="N32" t="s" s="2">
-        <v>325</v>
-      </c>
-      <c r="O32" t="s" s="2">
-        <v>326</v>
       </c>
       <c r="P32" t="s" s="2">
         <v>20</v>
@@ -5236,17 +5237,19 @@
         <v>20</v>
       </c>
       <c r="AB32" t="s" s="2">
-        <v>327</v>
-      </c>
-      <c r="AC32" s="2"/>
+        <v>20</v>
+      </c>
+      <c r="AC32" t="s" s="2">
+        <v>20</v>
+      </c>
       <c r="AD32" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AE32" t="s" s="2">
-        <v>116</v>
+        <v>20</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>78</v>
@@ -5264,10 +5267,10 @@
         <v>20</v>
       </c>
       <c r="AL32" t="s" s="2">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="AM32" t="s" s="2">
-        <v>329</v>
+        <v>263</v>
       </c>
       <c r="AN32" t="s" s="2">
         <v>20</v>
@@ -5275,23 +5278,21 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>320</v>
-      </c>
-      <c r="C33" t="s" s="2">
-        <v>331</v>
-      </c>
+        <v>325</v>
+      </c>
+      <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="H33" t="s" s="2">
         <v>20</v>
@@ -5303,19 +5304,19 @@
         <v>20</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="N33" t="s" s="2">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="O33" t="s" s="2">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="P33" t="s" s="2">
         <v>20</v>
@@ -5352,19 +5353,17 @@
         <v>20</v>
       </c>
       <c r="AB33" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AC33" t="s" s="2">
-        <v>20</v>
-      </c>
+        <v>332</v>
+      </c>
+      <c r="AC33" s="2"/>
       <c r="AD33" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AE33" t="s" s="2">
-        <v>20</v>
+        <v>116</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>78</v>
@@ -5382,10 +5381,10 @@
         <v>20</v>
       </c>
       <c r="AL33" t="s" s="2">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="AM33" t="s" s="2">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="AN33" t="s" s="2">
         <v>20</v>
@@ -5393,23 +5392,23 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="C34" t="s" s="2">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="D34" t="s" s="2">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G34" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="H34" t="s" s="2">
         <v>20</v>
@@ -5421,19 +5420,19 @@
         <v>20</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="N34" t="s" s="2">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="O34" t="s" s="2">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="P34" t="s" s="2">
         <v>20</v>
@@ -5482,7 +5481,7 @@
         <v>20</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>78</v>
@@ -5500,10 +5499,10 @@
         <v>20</v>
       </c>
       <c r="AL34" t="s" s="2">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="AM34" t="s" s="2">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="AN34" t="s" s="2">
         <v>20</v>
@@ -5511,20 +5510,20 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="C35" t="s" s="2">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="D35" t="s" s="2">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="G35" t="s" s="2">
         <v>79</v>
@@ -5539,19 +5538,19 @@
         <v>20</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="N35" t="s" s="2">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="O35" t="s" s="2">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="P35" t="s" s="2">
         <v>20</v>
@@ -5600,7 +5599,7 @@
         <v>20</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>78</v>
@@ -5618,10 +5617,10 @@
         <v>20</v>
       </c>
       <c r="AL35" t="s" s="2">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="AM35" t="s" s="2">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="AN35" t="s" s="2">
         <v>20</v>
@@ -5629,16 +5628,14 @@
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>320</v>
-      </c>
-      <c r="C36" t="s" s="2">
-        <v>340</v>
-      </c>
+        <v>341</v>
+      </c>
+      <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
-        <v>321</v>
+        <v>20</v>
       </c>
       <c r="E36" s="2"/>
       <c r="F36" t="s" s="2">
@@ -5657,20 +5654,18 @@
         <v>20</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>323</v>
+        <v>343</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>324</v>
+        <v>344</v>
       </c>
       <c r="N36" t="s" s="2">
-        <v>325</v>
-      </c>
-      <c r="O36" t="s" s="2">
-        <v>326</v>
-      </c>
+        <v>345</v>
+      </c>
+      <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
         <v>20</v>
       </c>
@@ -5718,7 +5713,7 @@
         <v>20</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>320</v>
+        <v>341</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>78</v>
@@ -5736,10 +5731,10 @@
         <v>20</v>
       </c>
       <c r="AL36" t="s" s="2">
-        <v>328</v>
+        <v>20</v>
       </c>
       <c r="AM36" t="s" s="2">
-        <v>329</v>
+        <v>346</v>
       </c>
       <c r="AN36" t="s" s="2">
         <v>20</v>
@@ -5747,14 +5742,14 @@
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
-        <v>20</v>
+        <v>348</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" t="s" s="2">
@@ -5770,21 +5765,21 @@
         <v>20</v>
       </c>
       <c r="J37" t="s" s="2">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>345</v>
-      </c>
-      <c r="N37" t="s" s="2">
-        <v>346</v>
-      </c>
-      <c r="O37" s="2"/>
+        <v>351</v>
+      </c>
+      <c r="N37" s="2"/>
+      <c r="O37" t="s" s="2">
+        <v>352</v>
+      </c>
       <c r="P37" t="s" s="2">
         <v>20</v>
       </c>
@@ -5832,7 +5827,7 @@
         <v>20</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>78</v>
@@ -5844,16 +5839,16 @@
         <v>20</v>
       </c>
       <c r="AJ37" t="s" s="2">
-        <v>102</v>
+        <v>353</v>
       </c>
       <c r="AK37" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL37" t="s" s="2">
-        <v>20</v>
+        <v>354</v>
       </c>
       <c r="AM37" t="s" s="2">
-        <v>347</v>
+        <v>334</v>
       </c>
       <c r="AN37" t="s" s="2">
         <v>20</v>
@@ -5861,21 +5856,21 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>348</v>
+        <v>355</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>348</v>
+        <v>355</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
-        <v>349</v>
+        <v>20</v>
       </c>
       <c r="E38" s="2"/>
       <c r="F38" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G38" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="H38" t="s" s="2">
         <v>20</v>
@@ -5884,21 +5879,19 @@
         <v>20</v>
       </c>
       <c r="J38" t="s" s="2">
-        <v>91</v>
+        <v>20</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>351</v>
+        <v>104</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>352</v>
+        <v>105</v>
       </c>
       <c r="N38" s="2"/>
-      <c r="O38" t="s" s="2">
-        <v>353</v>
-      </c>
+      <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
         <v>20</v>
       </c>
@@ -5946,28 +5939,28 @@
         <v>20</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>348</v>
+        <v>106</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH38" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="AI38" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AJ38" t="s" s="2">
-        <v>354</v>
+        <v>20</v>
       </c>
       <c r="AK38" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL38" t="s" s="2">
-        <v>355</v>
+        <v>20</v>
       </c>
       <c r="AM38" t="s" s="2">
-        <v>329</v>
+        <v>107</v>
       </c>
       <c r="AN38" t="s" s="2">
         <v>20</v>
@@ -5975,21 +5968,21 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
-        <v>20</v>
+        <v>109</v>
       </c>
       <c r="E39" s="2"/>
       <c r="F39" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G39" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="H39" t="s" s="2">
         <v>20</v>
@@ -6001,15 +5994,17 @@
         <v>20</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>357</v>
+        <v>110</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="N39" s="2"/>
+        <v>112</v>
+      </c>
+      <c r="N39" t="s" s="2">
+        <v>113</v>
+      </c>
       <c r="O39" s="2"/>
       <c r="P39" t="s" s="2">
         <v>20</v>
@@ -6058,19 +6053,19 @@
         <v>20</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH39" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="AI39" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AJ39" t="s" s="2">
-        <v>20</v>
+        <v>118</v>
       </c>
       <c r="AK39" t="s" s="2">
         <v>20</v>
@@ -6094,7 +6089,7 @@
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
-        <v>109</v>
+        <v>359</v>
       </c>
       <c r="E40" s="2"/>
       <c r="F40" t="s" s="2">
@@ -6107,24 +6102,26 @@
         <v>20</v>
       </c>
       <c r="I40" t="s" s="2">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="J40" t="s" s="2">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="K40" t="s" s="2">
         <v>110</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>111</v>
+        <v>360</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>112</v>
+        <v>361</v>
       </c>
       <c r="N40" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="O40" s="2"/>
+      <c r="O40" t="s" s="2">
+        <v>195</v>
+      </c>
       <c r="P40" t="s" s="2">
         <v>20</v>
       </c>
@@ -6172,7 +6169,7 @@
         <v>20</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>117</v>
+        <v>362</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>78</v>
@@ -6193,7 +6190,7 @@
         <v>20</v>
       </c>
       <c r="AM40" t="s" s="2">
-        <v>107</v>
+        <v>188</v>
       </c>
       <c r="AN40" t="s" s="2">
         <v>20</v>
@@ -6201,45 +6198,45 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
-        <v>360</v>
+        <v>20</v>
       </c>
       <c r="E41" s="2"/>
       <c r="F41" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G41" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="H41" t="s" s="2">
         <v>20</v>
       </c>
       <c r="I41" t="s" s="2">
-        <v>91</v>
+        <v>20</v>
       </c>
       <c r="J41" t="s" s="2">
-        <v>91</v>
+        <v>20</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>110</v>
+        <v>356</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="N41" t="s" s="2">
-        <v>113</v>
+        <v>366</v>
       </c>
       <c r="O41" t="s" s="2">
-        <v>195</v>
+        <v>367</v>
       </c>
       <c r="P41" t="s" s="2">
         <v>20</v>
@@ -6294,13 +6291,13 @@
         <v>78</v>
       </c>
       <c r="AH41" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="AI41" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AJ41" t="s" s="2">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="AK41" t="s" s="2">
         <v>20</v>
@@ -6309,7 +6306,7 @@
         <v>20</v>
       </c>
       <c r="AM41" t="s" s="2">
-        <v>188</v>
+        <v>368</v>
       </c>
       <c r="AN41" t="s" s="2">
         <v>20</v>
@@ -6317,10 +6314,10 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6328,7 +6325,7 @@
       </c>
       <c r="E42" s="2"/>
       <c r="F42" t="s" s="2">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="G42" t="s" s="2">
         <v>90</v>
@@ -6340,23 +6337,19 @@
         <v>20</v>
       </c>
       <c r="J42" t="s" s="2">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>357</v>
+        <v>370</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>366</v>
-      </c>
-      <c r="N42" t="s" s="2">
-        <v>367</v>
-      </c>
-      <c r="O42" t="s" s="2">
-        <v>368</v>
-      </c>
+        <v>372</v>
+      </c>
+      <c r="N42" s="2"/>
+      <c r="O42" s="2"/>
       <c r="P42" t="s" s="2">
         <v>20</v>
       </c>
@@ -6404,10 +6397,10 @@
         <v>20</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="AG42" t="s" s="2">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="AH42" t="s" s="2">
         <v>90</v>
@@ -6425,7 +6418,7 @@
         <v>20</v>
       </c>
       <c r="AM42" t="s" s="2">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="AN42" t="s" s="2">
         <v>20</v>
@@ -6433,18 +6426,18 @@
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
-        <v>20</v>
+        <v>375</v>
       </c>
       <c r="E43" s="2"/>
       <c r="F43" t="s" s="2">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="G43" t="s" s="2">
         <v>90</v>
@@ -6456,19 +6449,21 @@
         <v>20</v>
       </c>
       <c r="J43" t="s" s="2">
-        <v>91</v>
+        <v>20</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>371</v>
+        <v>356</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="N43" s="2"/>
-      <c r="O43" s="2"/>
+      <c r="O43" t="s" s="2">
+        <v>378</v>
+      </c>
       <c r="P43" t="s" s="2">
         <v>20</v>
       </c>
@@ -6516,10 +6511,10 @@
         <v>20</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="AG43" t="s" s="2">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="AH43" t="s" s="2">
         <v>90</v>
@@ -6534,10 +6529,10 @@
         <v>20</v>
       </c>
       <c r="AL43" t="s" s="2">
-        <v>20</v>
+        <v>379</v>
       </c>
       <c r="AM43" t="s" s="2">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="AN43" t="s" s="2">
         <v>20</v>
@@ -6545,21 +6540,21 @@
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
-        <v>376</v>
+        <v>20</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G44" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="H44" t="s" s="2">
         <v>20</v>
@@ -6571,18 +6566,16 @@
         <v>20</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>357</v>
+        <v>231</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="N44" s="2"/>
-      <c r="O44" t="s" s="2">
-        <v>379</v>
-      </c>
+      <c r="O44" s="2"/>
       <c r="P44" t="s" s="2">
         <v>20</v>
       </c>
@@ -6606,13 +6599,13 @@
         <v>20</v>
       </c>
       <c r="X44" t="s" s="2">
-        <v>20</v>
+        <v>155</v>
       </c>
       <c r="Y44" t="s" s="2">
-        <v>20</v>
+        <v>384</v>
       </c>
       <c r="Z44" t="s" s="2">
-        <v>20</v>
+        <v>385</v>
       </c>
       <c r="AA44" t="s" s="2">
         <v>20</v>
@@ -6630,13 +6623,13 @@
         <v>20</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH44" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="AI44" t="s" s="2">
         <v>20</v>
@@ -6648,10 +6641,10 @@
         <v>20</v>
       </c>
       <c r="AL44" t="s" s="2">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="AM44" t="s" s="2">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="AN44" t="s" s="2">
         <v>20</v>
@@ -6659,10 +6652,10 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -6685,16 +6678,20 @@
         <v>20</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>231</v>
+        <v>388</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>383</v>
+        <v>389</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>384</v>
-      </c>
-      <c r="N45" s="2"/>
-      <c r="O45" s="2"/>
+        <v>390</v>
+      </c>
+      <c r="N45" t="s" s="2">
+        <v>391</v>
+      </c>
+      <c r="O45" t="s" s="2">
+        <v>392</v>
+      </c>
       <c r="P45" t="s" s="2">
         <v>20</v>
       </c>
@@ -6718,13 +6715,13 @@
         <v>20</v>
       </c>
       <c r="X45" t="s" s="2">
-        <v>155</v>
+        <v>20</v>
       </c>
       <c r="Y45" t="s" s="2">
-        <v>385</v>
+        <v>20</v>
       </c>
       <c r="Z45" t="s" s="2">
-        <v>386</v>
+        <v>20</v>
       </c>
       <c r="AA45" t="s" s="2">
         <v>20</v>
@@ -6742,7 +6739,7 @@
         <v>20</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>78</v>
@@ -6760,128 +6757,12 @@
         <v>20</v>
       </c>
       <c r="AL45" t="s" s="2">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="AM45" t="s" s="2">
-        <v>387</v>
+        <v>393</v>
       </c>
       <c r="AN45" t="s" s="2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="s" s="2">
-        <v>388</v>
-      </c>
-      <c r="B46" t="s" s="2">
-        <v>388</v>
-      </c>
-      <c r="C46" s="2"/>
-      <c r="D46" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="E46" s="2"/>
-      <c r="F46" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G46" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="H46" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="I46" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="J46" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="K46" t="s" s="2">
-        <v>389</v>
-      </c>
-      <c r="L46" t="s" s="2">
-        <v>390</v>
-      </c>
-      <c r="M46" t="s" s="2">
-        <v>391</v>
-      </c>
-      <c r="N46" t="s" s="2">
-        <v>392</v>
-      </c>
-      <c r="O46" t="s" s="2">
-        <v>393</v>
-      </c>
-      <c r="P46" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="Q46" s="2"/>
-      <c r="R46" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="S46" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="T46" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="U46" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="V46" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="W46" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="X46" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="Y46" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="Z46" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AA46" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AB46" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AC46" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AD46" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AE46" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AF46" t="s" s="2">
-        <v>388</v>
-      </c>
-      <c r="AG46" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH46" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AI46" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AJ46" t="s" s="2">
-        <v>102</v>
-      </c>
-      <c r="AK46" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AL46" t="s" s="2">
-        <v>380</v>
-      </c>
-      <c r="AM46" t="s" s="2">
-        <v>394</v>
-      </c>
-      <c r="AN46" t="s" s="2">
         <v>20</v>
       </c>
     </row>

</xml_diff>